<commit_message>
Schedule Engine: Area → Building dimension from WBS (Pellet-1/2, Filtration)
- Buildings are taken from the WBS level holding building names (Additive
  Storage Shed, Green Pelletizing Building...), with the level above as the
  new Area / plant dimension; repeated names get the area added.
- Area dropdown, cascading Building dropdown with "Buildings from" level
  selector and area-name option; Area column, groupings, Easy Update,
  Timeline lanes, Setup, Ask and area-wise report tables.
- Demo rebuilt as Pellet Plant-1 / Pellet Plant-2 / Filtration Plant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H1BB9M3EwPpx4pEE5jFoAf
</commit_message>
<xml_diff>
--- a/schedule-engine/samples/Qty_Liquidation_Filled.xlsx
+++ b/schedule-engine/samples/Qty_Liquidation_Filled.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="126">
   <si>
     <t>Quantity tracker - items</t>
   </si>
@@ -86,13 +86,13 @@
     <t>Balance to erect</t>
   </si>
   <si>
-    <t>qmul0x900g5h</t>
+    <t>qmul33cej9ge</t>
   </si>
   <si>
     <t>Additive Grinding Building</t>
   </si>
   <si>
-    <t>Building structures</t>
+    <t>Pellet Plant-1</t>
   </si>
   <si>
     <t>Construction</t>
@@ -113,10 +113,13 @@
     <t>auto</t>
   </si>
   <si>
-    <t>qmul0x900o52</t>
-  </si>
-  <si>
-    <t>Screen House / Building</t>
+    <t>qmul33cej47p</t>
+  </si>
+  <si>
+    <t>Screen House</t>
+  </si>
+  <si>
+    <t>Pellet Plant-2</t>
   </si>
   <si>
     <t>Samal Brothers</t>
@@ -125,10 +128,13 @@
     <t>+ TS: equipment, crane &amp; conveyor supports</t>
   </si>
   <si>
-    <t>qmul0x90006w</t>
+    <t>qmul33cej833</t>
   </si>
   <si>
     <t>Return Fines Building</t>
+  </si>
+  <si>
+    <t>Filtration Plant</t>
   </si>
   <si>
     <t>Vrinda Bhillai (site fabrication)</t>
@@ -1066,13 +1072,13 @@
         <v>33</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>28</v>
@@ -1081,7 +1087,7 @@
         <v>1019</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J5" s="4">
         <v>1019</v>
@@ -1122,22 +1128,22 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>28</v>
@@ -1146,7 +1152,7 @@
         <v>393</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J6" s="4">
         <v>393</v>
@@ -1233,7 +1239,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1255,7 +1261,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1280,55 +1286,55 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1339,7 +1345,7 @@
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D4">
         <f>Items!H4-Items!K4</f>
@@ -1381,7 +1387,7 @@
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D5">
         <f>Items!H4-Items!L4</f>
@@ -1429,7 +1435,7 @@
         <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D6">
         <f>Items!H5-Items!K5</f>
@@ -1469,7 +1475,7 @@
         <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D7">
         <f>Items!H5-Items!L5</f>
@@ -1509,13 +1515,13 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D8">
         <f>Items!H6-Items!K6</f>
@@ -1549,13 +1555,13 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D9">
         <f>Items!H6-Items!L6</f>
@@ -1620,7 +1626,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1629,7 +1635,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1641,16 +1647,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1658,16 +1664,16 @@
         <v>23</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1675,16 +1681,16 @@
         <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1692,16 +1698,16 @@
         <v>23</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1709,16 +1715,16 @@
         <v>23</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1726,16 +1732,16 @@
         <v>23</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1743,16 +1749,16 @@
         <v>23</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1760,16 +1766,16 @@
         <v>32</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1777,16 +1783,16 @@
         <v>32</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1794,16 +1800,16 @@
         <v>32</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1811,16 +1817,16 @@
         <v>32</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1828,16 +1834,16 @@
         <v>32</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1845,16 +1851,16 @@
         <v>32</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1862,118 +1868,118 @@
         <v>32</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -2010,7 +2016,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2019,7 +2025,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2031,16 +2037,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2048,33 +2054,33 @@
         <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2104,7 +2110,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2116,7 +2122,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2128,28 +2134,28 @@
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2157,7 +2163,7 @@
         <v>24</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C4">
         <v>2000</v>
@@ -2172,10 +2178,10 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -2198,10 +2204,10 @@
         <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2224,10 +2230,10 @@
         <v>30</v>
       </c>
       <c r="G6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -2250,10 +2256,10 @@
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2261,7 +2267,7 @@
         <v>33</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C8">
         <v>1019</v>
@@ -2276,10 +2282,10 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -2302,10 +2308,10 @@
         <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -2328,18 +2334,18 @@
         <v>30</v>
       </c>
       <c r="G10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C11">
         <v>393</v>
@@ -2354,10 +2360,10 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2380,10 +2386,10 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2406,10 +2412,10 @@
         <v>30</v>
       </c>
       <c r="G13" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>